<commit_message>
feat: persist clothing items in PostgreSQL
</commit_message>
<xml_diff>
--- a/backend/exports/items.xlsx
+++ b/backend/exports/items.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,39 +466,78 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ca47d3d3-aa02-428e-bac0-478209192c5c</t>
+          <t>fe65df1d-73a3-4314-9497-8b5666573932</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>aa</t>
+          <t>string</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>string</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>blue</t>
+          <t>string</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>uploads\ca47d3d3-aa02-428e-bac0-478209192c5c_front_133921465173645984.jpg</t>
+          <t>uploads\fe65df1d-73a3-4314-9497-8b5666573932_front_133921465226938087.jpg</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>uploads\ca47d3d3-aa02-428e-bac0-478209192c5c_back_133921465226938087.jpg</t>
+          <t>uploads\fe65df1d-73a3-4314-9497-8b5666573932_back_133911093668301037.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>3a9fe41a-c8d7-472d-a09a-822229cedbc9</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>uploads\3a9fe41a-c8d7-472d-a09a-822229cedbc9_front_133911093668301037.jpg</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>uploads\3a9fe41a-c8d7-472d-a09a-822229cedbc9_back_133921465173645984.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add AI-generated captions for clothing items
</commit_message>
<xml_diff>
--- a/backend/exports/items.xlsx
+++ b/backend/exports/items.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,78 +466,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>fe65df1d-73a3-4314-9497-8b5666573932</t>
+          <t>b28db635-edcc-459e-8892-f920ede7e075</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>a</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>a</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aa
+</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>uploads\fe65df1d-73a3-4314-9497-8b5666573932_front_133921465226938087.jpg</t>
+          <t>uploads\b28db635-edcc-459e-8892-f920ede7e075_front_133921465173645984.jpg</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>uploads\fe65df1d-73a3-4314-9497-8b5666573932_back_133911093668301037.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>3a9fe41a-c8d7-472d-a09a-822229cedbc9</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>uploads\3a9fe41a-c8d7-472d-a09a-822229cedbc9_front_133911093668301037.jpg</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>uploads\3a9fe41a-c8d7-472d-a09a-822229cedbc9_back_133921465173645984.jpg</t>
+          <t>uploads\b28db635-edcc-459e-8892-f920ede7e075_back_133942081852602410.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>